<commit_message>
Evaluation Metrics columns added to moondream, llava_long, llava_short, qwen25vl_conf6
</commit_message>
<xml_diff>
--- a/demo/ic_demo_with_moondream.xlsx
+++ b/demo/ic_demo_with_moondream.xlsx
@@ -483,13 +483,13 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>5.669791110976001</v>
+        <v>5.67</v>
       </c>
       <c r="G2" t="n">
-        <v>0.2222222222222222</v>
+        <v>0.2222</v>
       </c>
       <c r="H2" t="n">
-        <v>0.2222222222222222</v>
+        <v>0.2222</v>
       </c>
     </row>
     <row r="3">
@@ -551,13 +551,13 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>21.46152503562546</v>
+        <v>21.46</v>
       </c>
       <c r="G4" t="n">
-        <v>0.5217391304347826</v>
+        <v>0.5217000000000001</v>
       </c>
       <c r="H4" t="n">
-        <v>0.5217391304347826</v>
+        <v>0.5217000000000001</v>
       </c>
     </row>
     <row r="5">
@@ -585,13 +585,13 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>15.61969968460128</v>
+        <v>15.62</v>
       </c>
       <c r="G5" t="n">
-        <v>0.3529411764705882</v>
+        <v>0.3529</v>
       </c>
       <c r="H5" t="n">
-        <v>0.3529411764705882</v>
+        <v>0.3529</v>
       </c>
     </row>
     <row r="6">
@@ -653,13 +653,13 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>2.75631563063758</v>
+        <v>2.76</v>
       </c>
       <c r="G7" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.2857</v>
       </c>
       <c r="H7" t="n">
-        <v>0.1904761904761905</v>
+        <v>0.1905</v>
       </c>
     </row>
     <row r="8">
@@ -687,7 +687,7 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>2.153749340017052</v>
+        <v>2.15</v>
       </c>
       <c r="G8" t="n">
         <v>0.3</v>
@@ -891,13 +891,13 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>0</v>
+        <v>1.37</v>
       </c>
       <c r="G14" t="n">
-        <v>0.1428571428571429</v>
+        <v>0.1429</v>
       </c>
       <c r="H14" t="n">
-        <v>0.1428571428571429</v>
+        <v>0.1429</v>
       </c>
     </row>
     <row r="15">
@@ -925,13 +925,13 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>6.567274736060395</v>
+        <v>6.57</v>
       </c>
       <c r="G15" t="n">
-        <v>0.1428571428571428</v>
+        <v>0.1429</v>
       </c>
       <c r="H15" t="n">
-        <v>0.1428571428571428</v>
+        <v>0.1429</v>
       </c>
     </row>
     <row r="16">
@@ -959,13 +959,13 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>8.295193507109859</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G16" t="n">
-        <v>0.3157894736842105</v>
+        <v>0.3158</v>
       </c>
       <c r="H16" t="n">
-        <v>0.2105263157894737</v>
+        <v>0.2105</v>
       </c>
     </row>
     <row r="17">
@@ -1027,7 +1027,7 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>6.528905536667997</v>
+        <v>6.53</v>
       </c>
       <c r="G18" t="n">
         <v>0.24</v>
@@ -1061,7 +1061,7 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>5.478531149356608</v>
+        <v>5.48</v>
       </c>
       <c r="G19" t="n">
         <v>0.1875</v>
@@ -1095,13 +1095,13 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>1.099621602822909</v>
+        <v>1.1</v>
       </c>
       <c r="G20" t="n">
-        <v>0.2222222222222222</v>
+        <v>0.2222</v>
       </c>
       <c r="H20" t="n">
-        <v>0.2222222222222222</v>
+        <v>0.2222</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Changes of scale in Evaluation metrics
</commit_message>
<xml_diff>
--- a/demo/ic_demo_with_moondream.xlsx
+++ b/demo/ic_demo_with_moondream.xlsx
@@ -486,10 +486,10 @@
         <v>5.67</v>
       </c>
       <c r="G2" t="n">
-        <v>0.2222</v>
+        <v>22.2222</v>
       </c>
       <c r="H2" t="n">
-        <v>0.2222</v>
+        <v>22.2222</v>
       </c>
     </row>
     <row r="3">
@@ -554,10 +554,10 @@
         <v>21.46</v>
       </c>
       <c r="G4" t="n">
-        <v>0.5217000000000001</v>
+        <v>52.1739</v>
       </c>
       <c r="H4" t="n">
-        <v>0.5217000000000001</v>
+        <v>52.1739</v>
       </c>
     </row>
     <row r="5">
@@ -588,10 +588,10 @@
         <v>15.62</v>
       </c>
       <c r="G5" t="n">
-        <v>0.3529</v>
+        <v>35.2941</v>
       </c>
       <c r="H5" t="n">
-        <v>0.3529</v>
+        <v>35.2941</v>
       </c>
     </row>
     <row r="6">
@@ -656,10 +656,10 @@
         <v>2.76</v>
       </c>
       <c r="G7" t="n">
-        <v>0.2857</v>
+        <v>28.5714</v>
       </c>
       <c r="H7" t="n">
-        <v>0.1905</v>
+        <v>19.0476</v>
       </c>
     </row>
     <row r="8">
@@ -690,10 +690,10 @@
         <v>2.15</v>
       </c>
       <c r="G8" t="n">
-        <v>0.3</v>
+        <v>30</v>
       </c>
       <c r="H8" t="n">
-        <v>0.1</v>
+        <v>10</v>
       </c>
     </row>
     <row r="9">
@@ -894,10 +894,10 @@
         <v>1.37</v>
       </c>
       <c r="G14" t="n">
-        <v>0.1429</v>
+        <v>14.2857</v>
       </c>
       <c r="H14" t="n">
-        <v>0.1429</v>
+        <v>14.2857</v>
       </c>
     </row>
     <row r="15">
@@ -928,10 +928,10 @@
         <v>6.57</v>
       </c>
       <c r="G15" t="n">
-        <v>0.1429</v>
+        <v>14.2857</v>
       </c>
       <c r="H15" t="n">
-        <v>0.1429</v>
+        <v>14.2857</v>
       </c>
     </row>
     <row r="16">
@@ -962,10 +962,10 @@
         <v>8.300000000000001</v>
       </c>
       <c r="G16" t="n">
-        <v>0.3158</v>
+        <v>31.5789</v>
       </c>
       <c r="H16" t="n">
-        <v>0.2105</v>
+        <v>21.0526</v>
       </c>
     </row>
     <row r="17">
@@ -1030,10 +1030,10 @@
         <v>6.53</v>
       </c>
       <c r="G18" t="n">
-        <v>0.24</v>
+        <v>24</v>
       </c>
       <c r="H18" t="n">
-        <v>0.24</v>
+        <v>24</v>
       </c>
     </row>
     <row r="19">
@@ -1064,10 +1064,10 @@
         <v>5.48</v>
       </c>
       <c r="G19" t="n">
-        <v>0.1875</v>
+        <v>18.75</v>
       </c>
       <c r="H19" t="n">
-        <v>0.1875</v>
+        <v>18.75</v>
       </c>
     </row>
     <row r="20">
@@ -1098,10 +1098,10 @@
         <v>1.1</v>
       </c>
       <c r="G20" t="n">
-        <v>0.2222</v>
+        <v>22.2222</v>
       </c>
       <c r="H20" t="n">
-        <v>0.2222</v>
+        <v>22.2222</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
One Shot, Few Shot, BertScore and ClipScore implemented
</commit_message>
<xml_diff>
--- a/demo/ic_demo_with_moondream.xlsx
+++ b/demo/ic_demo_with_moondream.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:J20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -457,6 +457,16 @@
           <t>ROUGE-L_F</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>BERTScore</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>CLIPScore</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -491,6 +501,12 @@
       <c r="H2" t="n">
         <v>22.2222</v>
       </c>
+      <c r="I2" t="n">
+        <v>29.14</v>
+      </c>
+      <c r="J2" t="n">
+        <v>25.93</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -525,6 +541,12 @@
       <c r="H3" t="n">
         <v>0</v>
       </c>
+      <c r="I3" t="n">
+        <v>26.61</v>
+      </c>
+      <c r="J3" t="n">
+        <v>22.29</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -559,6 +581,12 @@
       <c r="H4" t="n">
         <v>52.1739</v>
       </c>
+      <c r="I4" t="n">
+        <v>49.14</v>
+      </c>
+      <c r="J4" t="n">
+        <v>29.75</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -593,6 +621,12 @@
       <c r="H5" t="n">
         <v>35.2941</v>
       </c>
+      <c r="I5" t="n">
+        <v>46.41</v>
+      </c>
+      <c r="J5" t="n">
+        <v>21.56</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -615,17 +649,23 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Wearing glasses standing next to it</t>
+          <t>Paper, and a man wearing glasses holding a clipboard</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>4.99</v>
       </c>
       <c r="G6" t="n">
-        <v>0</v>
+        <v>22.2222</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>22.2222</v>
+      </c>
+      <c r="I6" t="n">
+        <v>34.37</v>
+      </c>
+      <c r="J6" t="n">
+        <v>20.85</v>
       </c>
     </row>
     <row r="7">
@@ -661,6 +701,12 @@
       <c r="H7" t="n">
         <v>19.0476</v>
       </c>
+      <c r="I7" t="n">
+        <v>14.54</v>
+      </c>
+      <c r="J7" t="n">
+        <v>21.9</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -695,6 +741,12 @@
       <c r="H8" t="n">
         <v>10</v>
       </c>
+      <c r="I8" t="n">
+        <v>29.22</v>
+      </c>
+      <c r="J8" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -717,17 +769,23 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Containers are used for heating water in industrial settings</t>
+          <t>Containers are used for heating water in a lab setting</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>1.54</v>
       </c>
       <c r="G9" t="n">
-        <v>0</v>
+        <v>7.4074</v>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>7.4074</v>
+      </c>
+      <c r="I9" t="n">
+        <v>27.09</v>
+      </c>
+      <c r="J9" t="n">
+        <v>26.59</v>
       </c>
     </row>
     <row r="10">
@@ -763,6 +821,12 @@
       <c r="H10" t="n">
         <v>0</v>
       </c>
+      <c r="I10" t="n">
+        <v>6.63</v>
+      </c>
+      <c r="J10" t="n">
+        <v>24.17</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -797,6 +861,12 @@
       <c r="H11" t="n">
         <v>0</v>
       </c>
+      <c r="I11" t="n">
+        <v>9.91</v>
+      </c>
+      <c r="J11" t="n">
+        <v>20.81</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -831,6 +901,12 @@
       <c r="H12" t="n">
         <v>0</v>
       </c>
+      <c r="I12" t="n">
+        <v>17.45</v>
+      </c>
+      <c r="J12" t="n">
+        <v>23.66</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -865,6 +941,12 @@
       <c r="H13" t="n">
         <v>0</v>
       </c>
+      <c r="I13" t="n">
+        <v>20.05</v>
+      </c>
+      <c r="J13" t="n">
+        <v>22.79</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -899,6 +981,12 @@
       <c r="H14" t="n">
         <v>14.2857</v>
       </c>
+      <c r="I14" t="n">
+        <v>18.33</v>
+      </c>
+      <c r="J14" t="n">
+        <v>22.92</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -921,17 +1009,23 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Containers on wheels in front of man</t>
+          <t>Containers on wheels in front of man; machine is gray, silver, black,</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>6.57</v>
+        <v>2.45</v>
       </c>
       <c r="G15" t="n">
-        <v>14.2857</v>
+        <v>10.5263</v>
       </c>
       <c r="H15" t="n">
-        <v>14.2857</v>
+        <v>10.5263</v>
+      </c>
+      <c r="I15" t="n">
+        <v>3.66</v>
+      </c>
+      <c r="J15" t="n">
+        <v>22.77</v>
       </c>
     </row>
     <row r="16">
@@ -967,6 +1061,12 @@
       <c r="H16" t="n">
         <v>21.0526</v>
       </c>
+      <c r="I16" t="n">
+        <v>46.87</v>
+      </c>
+      <c r="J16" t="n">
+        <v>20.06</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -989,7 +1089,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Containers on the table are made of metal</t>
+          <t>Containers on top of each other in front of building</t>
         </is>
       </c>
       <c r="F17" t="n">
@@ -1000,6 +1100,12 @@
       </c>
       <c r="H17" t="n">
         <v>0</v>
+      </c>
+      <c r="I17" t="n">
+        <v>6.84</v>
+      </c>
+      <c r="J17" t="n">
+        <v>17.26</v>
       </c>
     </row>
     <row r="18">
@@ -1023,17 +1129,23 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Containers on display in front of man in suit</t>
+          <t>Containers on display in front of white wall</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>6.53</v>
+        <v>5.89</v>
       </c>
       <c r="G18" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H18" t="n">
-        <v>24</v>
+        <v>25</v>
+      </c>
+      <c r="I18" t="n">
+        <v>33.22</v>
+      </c>
+      <c r="J18" t="n">
+        <v>20.37</v>
       </c>
     </row>
     <row r="19">
@@ -1057,7 +1169,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Containers on the floor in front of three men talking to each</t>
+          <t>Containers on the floor in front of three people talking to each</t>
         </is>
       </c>
       <c r="F19" t="n">
@@ -1069,6 +1181,12 @@
       <c r="H19" t="n">
         <v>18.75</v>
       </c>
+      <c r="I19" t="n">
+        <v>26.38</v>
+      </c>
+      <c r="J19" t="n">
+        <v>22.46</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1091,17 +1209,23 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Containers on the table in front of the men</t>
+          <t>Containers on the table in front of them</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>1.1</v>
+        <v>0.78</v>
       </c>
       <c r="G20" t="n">
-        <v>22.2222</v>
+        <v>17.1429</v>
       </c>
       <c r="H20" t="n">
-        <v>22.2222</v>
+        <v>17.1429</v>
+      </c>
+      <c r="I20" t="n">
+        <v>23.12</v>
+      </c>
+      <c r="J20" t="n">
+        <v>18.69</v>
       </c>
     </row>
   </sheetData>

</xml_diff>